<commit_message>
Updated CNN model, Slide deck and report
</commit_message>
<xml_diff>
--- a/Capstone_3/Notebooks/WBC_recognition_model_metrics.xlsx
+++ b/Capstone_3/Notebooks/WBC_recognition_model_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\goatf\Documents\Springboard\Capstone_3\Notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{585B435F-5E4B-4066-8F87-975AB26A37F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9D9BDB-3C7C-455D-9CA1-42D62964E987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C94E4085-2C7F-4CB3-B0A5-E535342E2A53}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="16">
   <si>
     <t>Precision</t>
   </si>
@@ -77,22 +77,13 @@
     <t>RBG KNN</t>
   </si>
   <si>
-    <t>GRAY SCALE KNN</t>
-  </si>
-  <si>
     <t>AUC</t>
   </si>
   <si>
     <t>RBG Random Forest</t>
   </si>
   <si>
-    <t>Tensor Flow</t>
-  </si>
-  <si>
-    <t>Tensor Flow GridSearch</t>
-  </si>
-  <si>
-    <t>5-k fold mean accuracy</t>
+    <t>CNN</t>
   </si>
 </sst>
 </file>
@@ -464,783 +455,472 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{186BF943-1AF4-489C-B75C-4DC5FA03CAE6}">
-  <dimension ref="A2:E53"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>13</v>
+      </c>
+    </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>0.66</v>
+      </c>
+      <c r="C2">
+        <v>0.23</v>
+      </c>
+      <c r="D2">
+        <v>0.34</v>
+      </c>
+      <c r="E2">
+        <v>0.75</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3">
-        <v>0.52</v>
+        <v>0.64</v>
       </c>
       <c r="C3">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="D3">
         <v>0.34</v>
       </c>
+      <c r="E3">
+        <v>0.86</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4">
-        <v>0.52</v>
+        <v>0.44</v>
       </c>
       <c r="C4">
-        <v>0.45</v>
+        <v>0.88</v>
       </c>
       <c r="D4">
-        <v>0.48</v>
+        <v>0.59</v>
+      </c>
+      <c r="E4">
+        <v>0.88</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5">
-        <v>0.4</v>
+        <v>0.67</v>
       </c>
       <c r="C5">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="D5">
-        <v>0.54</v>
+        <v>0.75</v>
+      </c>
+      <c r="E5">
+        <v>0.96</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6">
-        <v>0.78</v>
+        <v>0.43</v>
       </c>
       <c r="C6">
-        <v>0.79</v>
+        <v>0.68</v>
       </c>
       <c r="D6">
-        <v>0.78</v>
+        <v>0.53</v>
+      </c>
+      <c r="E6">
+        <v>0.88</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>0.43</v>
+        <v>0.89</v>
       </c>
       <c r="C7">
-        <v>0.55000000000000004</v>
+        <v>0.47</v>
       </c>
       <c r="D7">
-        <v>0.48</v>
+        <v>0.61</v>
+      </c>
+      <c r="E7">
+        <v>0.92</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8">
-        <v>0.89</v>
-      </c>
-      <c r="C8">
-        <v>0.31</v>
+        <v>9</v>
       </c>
       <c r="D8">
-        <v>0.46</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="B9">
+        <v>0.62</v>
+      </c>
+      <c r="C9">
+        <v>0.56000000000000005</v>
       </c>
       <c r="D9">
-        <v>0.51</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10">
-        <v>0.59</v>
+        <v>0.64</v>
       </c>
       <c r="C10">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="D10">
         <v>0.53</v>
-      </c>
-      <c r="D10">
-        <v>0.51</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11">
-        <v>0.6</v>
-      </c>
-      <c r="C11">
-        <v>0.51</v>
-      </c>
-      <c r="D11">
-        <v>0.49</v>
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B12" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" t="s">
-        <v>1</v>
-      </c>
-      <c r="D12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
+        <v>3</v>
+      </c>
+      <c r="B12">
+        <v>0.61</v>
+      </c>
+      <c r="C12">
+        <v>0.82</v>
+      </c>
+      <c r="D12">
+        <v>0.7</v>
+      </c>
+      <c r="E12">
+        <v>0.91</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B13">
-        <v>0.62</v>
+        <v>0.77</v>
       </c>
       <c r="C13">
-        <v>0.26</v>
+        <v>0.42</v>
       </c>
       <c r="D13">
-        <v>0.36</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="E13">
-        <v>0.44</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B14">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="C14">
-        <v>0.31</v>
+        <v>0.93</v>
       </c>
       <c r="D14">
-        <v>0.41</v>
+        <v>0.91</v>
       </c>
       <c r="E14">
-        <v>0.53</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B15">
-        <v>0.43</v>
+        <v>0.85</v>
       </c>
       <c r="C15">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="D15">
-        <v>0.57999999999999996</v>
+        <v>0.82</v>
       </c>
       <c r="E15">
-        <v>0.39</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B16">
-        <v>0.72</v>
+        <v>0.88</v>
       </c>
       <c r="C16">
-        <v>0.84</v>
+        <v>0.39</v>
       </c>
       <c r="D16">
-        <v>0.77</v>
+        <v>0.54</v>
       </c>
       <c r="E16">
-        <v>0.96</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B17">
-        <v>0.43</v>
+        <v>0.87</v>
       </c>
       <c r="C17">
-        <v>0.63</v>
+        <v>0.95</v>
       </c>
       <c r="D17">
-        <v>0.51</v>
+        <v>0.91</v>
       </c>
       <c r="E17">
-        <v>0.87</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>8</v>
-      </c>
-      <c r="B18">
-        <v>0.89</v>
-      </c>
-      <c r="C18">
-        <v>0.42</v>
+        <v>9</v>
       </c>
       <c r="D18">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="E18">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="B19">
+        <v>0.81</v>
+      </c>
+      <c r="C19">
+        <v>0.72</v>
       </c>
       <c r="D19">
-        <v>0.54</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B20">
-        <v>0.62</v>
+        <v>0.81</v>
       </c>
       <c r="C20">
-        <v>0.56000000000000005</v>
+        <v>0.79</v>
       </c>
       <c r="D20">
-        <v>0.45</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>11</v>
-      </c>
-      <c r="B21">
-        <v>0.63</v>
-      </c>
-      <c r="C21">
-        <v>0.54</v>
-      </c>
-      <c r="D21">
-        <v>0.53</v>
+        <v>15</v>
+      </c>
+      <c r="B21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>2</v>
+      </c>
+      <c r="E21" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22" t="s">
-        <v>1</v>
-      </c>
-      <c r="D22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E22" t="s">
-        <v>14</v>
+        <v>4</v>
+      </c>
+      <c r="B22">
+        <v>0.94</v>
+      </c>
+      <c r="C22">
+        <v>0.79</v>
+      </c>
+      <c r="D22">
+        <v>0.86</v>
+      </c>
+      <c r="E22">
+        <v>0.97</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B23">
-        <v>0.61</v>
+        <v>0.95</v>
       </c>
       <c r="C23">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="D23">
-        <v>0.69</v>
+        <v>0.95</v>
       </c>
       <c r="E23">
-        <v>0.42</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B24">
-        <v>0.75</v>
+        <v>0.99</v>
       </c>
       <c r="C24">
-        <v>0.42</v>
+        <v>0.99</v>
       </c>
       <c r="D24">
-        <v>0.54</v>
+        <v>0.99</v>
       </c>
       <c r="E24">
-        <v>0.67</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B25">
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
       <c r="C25">
-        <v>0.93</v>
+        <v>0.98</v>
       </c>
       <c r="D25">
-        <v>0.9</v>
+        <v>0.87</v>
       </c>
       <c r="E25">
-        <v>0.35</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B26">
-        <v>0.87</v>
+        <v>0.76</v>
       </c>
       <c r="C26">
-        <v>0.81</v>
+        <v>0.91</v>
       </c>
       <c r="D26">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="E26">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B27">
-        <v>0.87</v>
+        <v>0.97</v>
       </c>
       <c r="C27">
-        <v>0.39</v>
+        <v>0.95</v>
       </c>
       <c r="D27">
-        <v>0.54</v>
+        <v>0.96</v>
       </c>
       <c r="E27">
-        <v>0.95</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28">
-        <v>0.86</v>
-      </c>
-      <c r="C28">
-        <v>0.95</v>
+        <v>10</v>
       </c>
       <c r="D28">
-        <v>0.9</v>
-      </c>
-      <c r="E28">
-        <v>0.99</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="B29">
+        <v>0.9</v>
+      </c>
+      <c r="C29">
+        <v>0.93</v>
       </c>
       <c r="D29">
-        <v>0.79</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>10</v>
-      </c>
       <c r="B30">
-        <v>0.81</v>
+        <v>0.93</v>
       </c>
       <c r="C30">
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
       <c r="D30">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31">
-        <v>0.8</v>
-      </c>
-      <c r="C31">
-        <v>0.79</v>
-      </c>
-      <c r="D31">
-        <v>0.78</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" t="s">
-        <v>0</v>
-      </c>
-      <c r="C32" t="s">
-        <v>1</v>
-      </c>
-      <c r="D32" t="s">
-        <v>2</v>
-      </c>
-      <c r="E32" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>3</v>
-      </c>
-      <c r="B33">
-        <v>0.65</v>
-      </c>
-      <c r="C33">
-        <v>0.49</v>
-      </c>
-      <c r="D33">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="E33">
-        <v>0.88</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>4</v>
-      </c>
-      <c r="B34">
-        <v>0.62</v>
-      </c>
-      <c r="C34">
-        <v>0.63</v>
-      </c>
-      <c r="D34">
-        <v>0.62</v>
-      </c>
-      <c r="E34">
-        <v>0.94</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>5</v>
-      </c>
-      <c r="B35">
-        <v>0.91</v>
-      </c>
-      <c r="C35">
-        <v>0.8</v>
-      </c>
-      <c r="D35">
-        <v>0.85</v>
-      </c>
-      <c r="E35">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>6</v>
-      </c>
-      <c r="B36">
-        <v>0.81</v>
-      </c>
-      <c r="C36">
-        <v>0.82</v>
-      </c>
-      <c r="D36">
-        <v>0.81</v>
-      </c>
-      <c r="E36">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>7</v>
-      </c>
-      <c r="B37">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="C37">
-        <v>0.79</v>
-      </c>
-      <c r="D37">
-        <v>0.65</v>
-      </c>
-      <c r="E37">
-        <v>0.94</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>8</v>
-      </c>
-      <c r="B38">
-        <v>0.81</v>
-      </c>
-      <c r="C38">
-        <v>0.91</v>
-      </c>
-      <c r="D38">
-        <v>0.85</v>
-      </c>
-      <c r="E38">
-        <v>0.97</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>9</v>
-      </c>
-      <c r="D39">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>10</v>
-      </c>
-      <c r="B40">
-        <v>0.72</v>
-      </c>
-      <c r="C40">
-        <v>0.74</v>
-      </c>
-      <c r="D40">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>11</v>
-      </c>
-      <c r="B41">
-        <v>0.75</v>
-      </c>
-      <c r="C41">
-        <v>0.74</v>
-      </c>
-      <c r="D41">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>18</v>
-      </c>
-      <c r="B42">
-        <v>0.62390000000000001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>17</v>
-      </c>
-      <c r="B43" t="s">
-        <v>0</v>
-      </c>
-      <c r="C43" t="s">
-        <v>1</v>
-      </c>
-      <c r="D43" t="s">
-        <v>2</v>
-      </c>
-      <c r="E43" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>3</v>
-      </c>
-      <c r="B44">
-        <v>0.79</v>
-      </c>
-      <c r="C44">
-        <v>0.3</v>
-      </c>
-      <c r="D44">
-        <v>0.4</v>
-      </c>
-      <c r="E44">
-        <v>0.91</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>4</v>
-      </c>
-      <c r="B45">
-        <v>0.44</v>
-      </c>
-      <c r="C45">
-        <v>0.84</v>
-      </c>
-      <c r="D45">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="E45">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>5</v>
-      </c>
-      <c r="B46">
-        <v>0.89</v>
-      </c>
-      <c r="C46">
-        <v>0.93</v>
-      </c>
-      <c r="D46">
-        <v>0.91</v>
-      </c>
-      <c r="E46">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>6</v>
-      </c>
-      <c r="B47">
-        <v>0.84</v>
-      </c>
-      <c r="C47">
-        <v>0.81</v>
-      </c>
-      <c r="D47">
-        <v>0.83</v>
-      </c>
-      <c r="E47">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>7</v>
-      </c>
-      <c r="B48">
-        <v>0.54</v>
-      </c>
-      <c r="C48">
-        <v>0.9</v>
-      </c>
-      <c r="D48">
-        <v>0.67</v>
-      </c>
-      <c r="E48">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49">
         <v>0.92</v>
-      </c>
-      <c r="C49">
-        <v>0.83</v>
-      </c>
-      <c r="D49">
-        <v>0.87</v>
-      </c>
-      <c r="E49">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>9</v>
-      </c>
-      <c r="D50">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>10</v>
-      </c>
-      <c r="B51">
-        <v>0.74</v>
-      </c>
-      <c r="C51">
-        <v>0.77</v>
-      </c>
-      <c r="D51">
-        <v>0.72</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>11</v>
-      </c>
-      <c r="B52">
-        <v>0.79</v>
-      </c>
-      <c r="C52">
-        <v>0.74</v>
-      </c>
-      <c r="D52">
-        <v>0.73</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>18</v>
-      </c>
-      <c r="B53">
-        <v>0.78810000000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>